<commit_message>
bug fix with bg job
</commit_message>
<xml_diff>
--- a/v2/agents/expense-calc/workspace/Expenses_History.xlsx
+++ b/v2/agents/expense-calc/workspace/Expenses_History.xlsx
@@ -17,6 +17,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06-13" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06-10" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06-09" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06-08" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06-07" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06-06" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06-04" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06-03" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06-02" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-05-31" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -456,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,108 +495,108 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46182</v>
+        <v>46173</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11:01:44</t>
+          <t>12:24:08</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>APPLE.COM/BILL</t>
+          <t>MIDJOURNEY INC.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Subscriptions &amp; Digital</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1680</v>
+        <v>1823</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46182</v>
+        <v>46173</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>16:02:25</t>
+          <t>17:47:23</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>OPENART AI</t>
+          <t>MITSUIFUDOUSANGURU-PUUNEI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Subscriptions &amp; Digital</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2311</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46183</v>
+        <v>46173</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>14:41:32</t>
+          <t>19:34:34</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AMAZON CO JP</t>
+          <t>STARBUCKS COFFEE JAPAN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Shopping &amp; Amenities</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2832</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46183</v>
+        <v>46173</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>16:56:46</t>
+          <t>23:33:32</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SOFTBANKM</t>
+          <t>SEVEN-ELEVEN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Utilities &amp; Phone</t>
+          <t>Food &amp; Convenience</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>12455</v>
+        <v>3325</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46186</v>
+        <v>46175</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10:52:28</t>
+          <t>02:18:11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>OPENAI *CHATGPT SUBSCR</t>
+          <t>GOOGLE*CLOUD VJKBV3</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -598,21 +605,21 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3670</v>
+        <v>153</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46186</v>
+        <v>46175</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>19:03:36</t>
+          <t>07:19:09</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TECTKITIJYOUZITENN</t>
+          <t>Amazon Web Services</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -621,136 +628,136 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>14800</v>
+        <v>4183</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46187</v>
+        <v>46175</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>00:10:41</t>
+          <t>17:57:19</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>SEVEN-ELEVEN</t>
+          <t>Amazon Web Services</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Food &amp; Convenience</t>
+          <t>Shopping &amp; Amenities</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2351</v>
+        <v>752</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46187</v>
+        <v>46175</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>00:13:46</t>
+          <t>19:34:32</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>FAMILYMART</t>
+          <t>UBER * EATS PENDING</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Food &amp; Convenience</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>555</v>
+        <v>1771</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46187</v>
+        <v>46176</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>20:31:04</t>
+          <t>13:59:20</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DEIRI-YAMAZAKI</t>
+          <t>MODAL.COM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Food &amp; Convenience</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>819</v>
+        <v>2668</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46187</v>
+        <v>46177</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>23:39:07</t>
+          <t>02:51:32</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>RAKUTEN KOBO</t>
+          <t>AMAZON CO JP</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Subscriptions &amp; Digital</t>
+          <t>Shopping &amp; Amenities</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>594</v>
+        <v>1930</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46188</v>
+        <v>46179</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>13:03:31</t>
+          <t>17:28:40</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OPENART AI</t>
+          <t>MARUETSU KANAMACHI</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Subscriptions &amp; Digital</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2335</v>
+        <v>3500</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46189</v>
+        <v>46180</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>21:52:05</t>
+          <t>09:07:07</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CURSOR, AI POWERED IDE</t>
+          <t>OPENAI *CHATGPT SUBSCR</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -759,44 +766,44 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3193</v>
+        <v>3669</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46191</v>
+        <v>46180</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>22:57:04</t>
+          <t>19:46:25</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>AMAZON CO JP</t>
+          <t>DEIRI-YAMAZAKI</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Shopping &amp; Amenities</t>
+          <t>Food &amp; Convenience</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>1141</v>
+        <v>2147</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46194</v>
+        <v>46180</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>17:23:54</t>
+          <t>20:57:29</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MERCARI</t>
+          <t>AMAZON CO JP</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -805,44 +812,44 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>34800</v>
+        <v>440</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46194</v>
+        <v>46181</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>18:05:27</t>
+          <t>19:48:10</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>OPENAI</t>
+          <t>FAMILYMART</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Subscriptions &amp; Digital</t>
+          <t>Food &amp; Convenience</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>1848</v>
+        <v>614</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46194</v>
+        <v>46182</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>18:47:04</t>
+          <t>11:01:44</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>OPENAI</t>
+          <t>APPLE.COM/BILL</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -851,52 +858,397 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>1774</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46194</v>
+        <v>46182</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>19:51:50</t>
+          <t>16:02:25</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>FAMILYMART</t>
+          <t>OPENART AI</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Food &amp; Convenience</t>
+          <t>Subscriptions &amp; Digital</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2421</v>
+        <v>2311</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>14:41:32</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AMAZON CO JP</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>2832</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>16:56:46</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>SOFTBANKM</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Utilities &amp; Phone</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>12455</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>10:52:28</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>OPENAI *CHATGPT SUBSCR</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Subscriptions &amp; Digital</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>3670</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>46186</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>19:03:36</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TECTKITIJYOUZITENN</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>14800</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>00:10:41</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>SEVEN-ELEVEN</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Food &amp; Convenience</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>2351</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>00:13:46</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>FAMILYMART</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Food &amp; Convenience</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>20:31:04</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>DEIRI-YAMAZAKI</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Food &amp; Convenience</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46187</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>23:39:07</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>RAKUTEN KOBO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Subscriptions &amp; Digital</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46188</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>13:03:31</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>OPENART AI</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Subscriptions &amp; Digital</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>2335</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>21:52:05</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>CURSOR, AI POWERED IDE</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Subscriptions &amp; Digital</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>3193</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>22:57:04</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>AMAZON CO JP</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1141</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>17:23:54</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MERCARI</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>34800</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>18:05:27</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>OPENAI</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Subscriptions &amp; Digital</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>18:47:04</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>OPENAI</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Subscriptions &amp; Digital</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1774</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46194</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>19:51:50</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>FAMILYMART</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Food &amp; Convenience</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>2421</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
         <v>46195</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>00:43:14</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>GOOGLE*GOOGLE ONE</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Subscriptions &amp; Digital</t>
         </is>
       </c>
-      <c r="E19" t="n">
+      <c r="E34" t="n">
         <v>2900</v>
       </c>
     </row>
@@ -1003,6 +1355,708 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Merchant</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Amount_JPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>19:48:10</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FAMILYMART</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Food &amp; Convenience</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>614</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Merchant</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Amount_JPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>09:07:07</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>OPENAI *CHATGPT SUBSCR</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Subscriptions &amp; Digital</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>3669</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>19:46:25</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>DEIRI-YAMAZAKI</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Food &amp; Convenience</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2147</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46180</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>20:57:29</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>AMAZON CO JP</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>6256</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Merchant</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Amount_JPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46179</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>17:28:40</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MARUETSU KANAMACHI</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>3500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Merchant</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Amount_JPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>02:51:32</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AMAZON CO JP</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1930</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1930</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Merchant</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Amount_JPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46176</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>13:59:20</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MODAL.COM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2668</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2668</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Merchant</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Amount_JPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>02:18:11</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>GOOGLE*CLOUD VJKBV3</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Subscriptions &amp; Digital</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>07:19:09</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>4183</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>17:57:19</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Shopping &amp; Amenities</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>19:34:32</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>UBER * EATS PENDING</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1771</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>6859</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Merchant</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Amount_JPY</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>12:24:08</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MIDJOURNEY INC.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>17:47:23</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MITSUIFUDOUSANGURU-PUUNEI</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>19:34:34</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>STARBUCKS COFFEE JAPAN</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>23:33:32</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>SEVEN-ELEVEN</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Food &amp; Convenience</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>3325</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>7809</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>